<commit_message>
correct aphia_ids, add contributors and improve documentation
</commit_message>
<xml_diff>
--- a/inst/extdata/Mesozooplankton_Kattegat_Skagerrak_taxa_and_biomass_calculations.xlsx
+++ b/inst/extdata/Mesozooplankton_Kattegat_Skagerrak_taxa_and_biomass_calculations.xlsx
@@ -794,7 +794,7 @@
         <v>15</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>345919</v>
+        <v>104249</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="9" t="n">
@@ -830,7 +830,7 @@
         <v>15</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>149755</v>
+        <v>104251</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="9" t="n">
@@ -866,7 +866,7 @@
         <v>15</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>346037</v>
+        <v>104257</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="9" t="n">
@@ -1189,7 +1189,7 @@
         <v>40</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>106415</v>
+        <v>1101</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="9" t="n">
@@ -1409,7 +1409,7 @@
         <v>15</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>103407</v>
+        <v>1770057</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="9" t="n">

</xml_diff>